<commit_message>
BackUp Kft. árlistája és az ügyfelünk CodeLinks Kft. árajánlata Excel táblázatokban
</commit_message>
<xml_diff>
--- a/BackUp Kft. ÁRLISTA.xlsx
+++ b/BackUp Kft. ÁRLISTA.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kralj\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E49D067-6A0A-46D5-A08A-B4D365A280A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{622C96A8-A016-4953-AD6C-68B59564687D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{69C008BB-116E-4B9E-837F-96DF98BB6AE9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="40">
   <si>
     <t>Eszköz típusa</t>
   </si>
@@ -50,12 +50,6 @@
     <t>4.200.000 Ft</t>
   </si>
   <si>
-    <t>1.800.000 Ft</t>
-  </si>
-  <si>
-    <t>6.000.000 Ft</t>
-  </si>
-  <si>
     <t>Összesen:</t>
   </si>
   <si>
@@ -68,21 +62,9 @@
     <t>C9800-L-C-K9</t>
   </si>
   <si>
-    <t>C9115AXE-E x3</t>
-  </si>
-  <si>
-    <t>1.150.000 Ft</t>
-  </si>
-  <si>
     <t>900.000 Ft</t>
   </si>
   <si>
-    <t>210 000 Ft x3</t>
-  </si>
-  <si>
-    <t>90 000 Ft x3</t>
-  </si>
-  <si>
     <t>219 600Ft</t>
   </si>
   <si>
@@ -101,27 +83,9 @@
     <t>Wireless LAN Controller</t>
   </si>
   <si>
-    <t>C9200L-24T-4G-E</t>
-  </si>
-  <si>
-    <t>401 368,00 Ft x3</t>
-  </si>
-  <si>
-    <t>127 708,00 Ft x3</t>
-  </si>
-  <si>
-    <t>1 587 228 Ft</t>
-  </si>
-  <si>
-    <t>2 487 000 Ft</t>
-  </si>
-  <si>
     <t>Windows Server 2022 Standard</t>
   </si>
   <si>
-    <t>2 827 719 Ft</t>
-  </si>
-  <si>
     <t>Dell PowerEdge R450</t>
   </si>
   <si>
@@ -138,15 +102,68 @@
   </si>
   <si>
     <t>Kábelek</t>
+  </si>
+  <si>
+    <t>210.000 Ft</t>
+  </si>
+  <si>
+    <t>400.000 Ft</t>
+  </si>
+  <si>
+    <t>500.000 Ft</t>
+  </si>
+  <si>
+    <t>1.700.000 Ft</t>
+  </si>
+  <si>
+    <t>800.000 Ft</t>
+  </si>
+  <si>
+    <t>32.845.540 Ft</t>
+  </si>
+  <si>
+    <t>C9115AXE-E</t>
+  </si>
+  <si>
+    <t>1.200.000 Ft</t>
+  </si>
+  <si>
+    <t>65.000 Ft</t>
+  </si>
+  <si>
+    <t>Cisco C9200L-24P-4X-E</t>
+  </si>
+  <si>
+    <t>250.000 Ft</t>
+  </si>
+  <si>
+    <t>850.000 Ft</t>
+  </si>
+  <si>
+    <t>1.642.277 Ft</t>
+  </si>
+  <si>
+    <t>10.200.000 Ft</t>
+  </si>
+  <si>
+    <t>3.300.000 Ft</t>
+  </si>
+  <si>
+    <t>825.000 Ft</t>
+  </si>
+  <si>
+    <t>51.090.140 Ft</t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="6" formatCode="#,##0\ &quot;Ft&quot;;[Red]\-#,##0\ &quot;Ft&quot;"/>
-    <numFmt numFmtId="173" formatCode="#,##0\ &quot;Ft&quot;"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0\ &quot;Ft&quot;;[Red]\-#,##0\ &quot;Ft&quot;"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -185,24 +202,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <i/>
-      <u/>
-      <sz val="28"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
-      <sz val="22"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -230,6 +229,23 @@
       <name val="Aptos Display"/>
       <family val="2"/>
       <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="26"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="20"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -246,7 +262,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -270,50 +286,9 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
-      <bottom style="thin">
-        <color theme="0" tint="-0.14999847407452621"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color theme="0" tint="-0.14999847407452621"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="0" tint="-0.14999847407452621"/>
-      </right>
-      <top style="thin">
-        <color theme="0" tint="-0.14999847407452621"/>
-      </top>
       <bottom style="thin">
         <color theme="0" tint="-0.14999847407452621"/>
       </bottom>
@@ -335,155 +310,70 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
+      <left/>
+      <right style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color theme="0" tint="-0.14999847407452621"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color theme="0" tint="-0.14999847407452621"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="6" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="6" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="6" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="6" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="6" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="6" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="173" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="6" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normál" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -499,7 +389,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office-téma">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -826,167 +716,171 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+    </row>
+    <row r="5" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="F5" s="8"/>
+      <c r="G5" s="1"/>
+    </row>
+    <row r="6" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" s="13" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+      <c r="C6" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" s="8"/>
+      <c r="G6" s="1"/>
+    </row>
+    <row r="7" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" s="20" t="s">
+      <c r="C8" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="7" t="s">
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="14" t="s">
         <v>9</v>
-      </c>
-      <c r="C4" s="17">
-        <v>750000</v>
-      </c>
-      <c r="D4" s="17">
-        <v>400000</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="5"/>
-      <c r="G4" s="2"/>
-    </row>
-    <row r="5" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="6"/>
-      <c r="G5" s="1"/>
-    </row>
-    <row r="6" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="25" t="s">
-        <v>30</v>
-      </c>
-      <c r="B6" s="22" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" s="30">
-        <v>388000</v>
-      </c>
-      <c r="D6" s="27"/>
-      <c r="E6" s="28">
-        <f>20*C6</f>
-        <v>7760000</v>
-      </c>
-      <c r="F6" s="6"/>
-      <c r="G6" s="1"/>
-    </row>
-    <row r="7" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="B7" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" s="26">
-        <v>1642277</v>
-      </c>
-      <c r="D7" s="9"/>
-      <c r="E7" s="31">
-        <f>20*C7</f>
-        <v>32845540</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" s="16">
-        <v>1700000</v>
-      </c>
-      <c r="D8" s="21" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" s="18" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="B9" s="23"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="14" t="s">
-        <v>15</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" spans="1:7" ht="36" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="E10" s="19">
-        <f>SUM(E2:E9)</f>
-        <v>40605540</v>
-      </c>
-      <c r="F10" s="1"/>
+    <row r="10" spans="1:7" ht="34.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="F10" s="17"/>
       <c r="G10" s="1"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -995,22 +889,22 @@
     </row>
     <row r="19" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="20" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E20" s="10"/>
+      <c r="E20" s="5"/>
     </row>
     <row r="23" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="10"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
     </row>
     <row r="25" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B25" s="10"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="10"/>
+      <c r="B25" s="5"/>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="7" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Hozzáadtam a szerverfarmon elhelyezett szerver árát is, mert az kimaradt
</commit_message>
<xml_diff>
--- a/BackUp Kft. ÁRLISTA.xlsx
+++ b/BackUp Kft. ÁRLISTA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{622C96A8-A016-4953-AD6C-68B59564687D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2BAB938-3C59-4FE1-BFDE-476B0BCEFB9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{69C008BB-116E-4B9E-837F-96DF98BB6AE9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="43">
   <si>
     <t>Eszköz típusa</t>
   </si>
@@ -92,12 +92,6 @@
     <t xml:space="preserve">Dell PowerEdge R640 (10XSFF) </t>
   </si>
   <si>
-    <t>Storage Szerver (2x)</t>
-  </si>
-  <si>
-    <t>Storage Szerver (20x)</t>
-  </si>
-  <si>
     <t>Samsung SSD PM1653</t>
   </si>
   <si>
@@ -116,9 +110,6 @@
     <t>1.700.000 Ft</t>
   </si>
   <si>
-    <t>800.000 Ft</t>
-  </si>
-  <si>
     <t>32.845.540 Ft</t>
   </si>
   <si>
@@ -152,10 +143,28 @@
     <t>825.000 Ft</t>
   </si>
   <si>
-    <t>51.090.140 Ft</t>
-  </si>
-  <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>Storage Szerver (3x)</t>
+  </si>
+  <si>
+    <t>SSD (20x)</t>
+  </si>
+  <si>
+    <t>HDD (10x)</t>
+  </si>
+  <si>
+    <t>Seagate Exos X24 16TB</t>
+  </si>
+  <si>
+    <t>238.890 Ft</t>
+  </si>
+  <si>
+    <t>2.388.900 Ft</t>
+  </si>
+  <si>
+    <t>53.879.040 Ft</t>
   </si>
 </sst>
 </file>
@@ -326,7 +335,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -352,18 +361,8 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
@@ -719,16 +718,16 @@
       <c r="A1" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="9" t="s">
         <v>1</v>
       </c>
     </row>
@@ -736,51 +735,51 @@
       <c r="A2" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="12" t="s">
-        <v>35</v>
+      <c r="E2" s="10" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" s="12" t="s">
+      <c r="B3" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" s="10" t="s">
         <v>33</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="E4" s="12" t="s">
-        <v>29</v>
+      <c r="C4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>26</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -789,35 +788,35 @@
       <c r="A5" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>37</v>
+      <c r="B5" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>34</v>
       </c>
       <c r="F5" s="8"/>
       <c r="G5" s="1"/>
     </row>
     <row r="6" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="E6" s="15" t="s">
+      <c r="C6" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>26</v>
       </c>
       <c r="F6" s="8"/>
@@ -825,65 +824,80 @@
     </row>
     <row r="7" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="D7" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="E7" s="15" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8" s="15" t="s">
-        <v>25</v>
+      <c r="C8" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="14" t="s">
-        <v>9</v>
+        <v>15</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>23</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" spans="1:7" ht="34.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="18" t="s">
-        <v>4</v>
+    <row r="10" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
-      <c r="E10" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="F10" s="17"/>
+      <c r="E10" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="F10" s="13"/>
       <c r="G10" s="1"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="34.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="15" t="s">
+        <v>42</v>
+      </c>
       <c r="F11" s="3"/>
       <c r="G11" s="4"/>
     </row>

</xml_diff>